<commit_message>
Rebuild Week Apr8-Apr15 sheet matching template format (flat table, colored badges)
</commit_message>
<xml_diff>
--- a/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
+++ b/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,8 +80,26 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -142,6 +160,36 @@
         <bgColor rgb="007030A0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A103C"/>
+        <bgColor rgb="001A103C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEE2E6"/>
+        <bgColor rgb="00DEE2E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D6EFD"/>
+        <bgColor rgb="000D6EFD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FD7E14"/>
+        <bgColor rgb="00FD7E14"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006F42C1"/>
+        <bgColor rgb="006F42C1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -176,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -211,6 +259,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2606,1037 +2661,747 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="9" min="1" max="1"/>
-    <col width="55" customWidth="1" style="9" min="2" max="2"/>
-    <col width="12" customWidth="1" style="9" min="3" max="3"/>
-    <col width="15" customWidth="1" style="9" min="4" max="4"/>
+    <col width="12" customWidth="1" style="9" min="1" max="1"/>
+    <col width="13" customWidth="1" style="9" min="2" max="2"/>
+    <col width="70" customWidth="1" style="9" min="3" max="3"/>
+    <col width="12" customWidth="1" style="9" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>AI 1st SEO — Weekly Tasks: April 8-15, 2026</t>
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>AI 1st SEO — Weekly Tasks (April 8 - April 15, 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Dev 1 — Deepthi Gunda (AI/ML &amp; GEO Engine)</t>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NEW (from Guide/WBS)</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>GEO Scanner: Add 5 new AI-readiness criteria to probe engine (WBS 1.3 — target 25 total GEO criteria)</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>WBS 1.3</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>GEO Scanner: Add 5 new AI-readiness criteria to probe engine (target: 25 total GEO criteria)</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Investigate and document how business directory data is ingested into DynamoDB — prepare backend walkthrough for next meeting</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Ensure all GEO routes work on Lambda after DynamoDB migration (test geo-probe/models, aeo/analyze, chatbot/session)</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Prepare demo of business directory backend + data ingestion process for next Tuesday meeting</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Work with Amira on documenting the search/scraping pipeline for the AI Business Directory</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Prepare to present backend details and search process at next meeting</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>Technical SEO Executor: Build auto-fix for sitemap.xml generation from scan results (WBS 2.1)</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>Verify content-briefs and content-score endpoints work with DynamoDB (db_dynamo.py fallback)</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>Merge dev2-samar-merge branch to main if not already done</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>Research two-way email send/receive solutions (SES vs ImprovMX vs iCloud) — report findings by Tuesday</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>Provide iCloud email settings to Gurbachan for official business email setup</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Send Gurbachan the automation hub / content generation demo link for review</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>Developer API: Document all 45+ API endpoints with request/response examples for team reference (WBS 6.2)</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>DynamoDB migration complete — monitor for any endpoint errors post-deploy</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>OpenClaw Gateway installed — wire up Phase 1 integration (report delivery via /hooks/agent)</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLEANUP (carryover)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>Investigate and document how business directory data is ingested into DynamoDB — prepare backend walkthrough for next meeting</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>From Zoom</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Ensure all GEO routes work on Lambda after DynamoDB migration (test geo-probe/models, aeo/analyze, chatbot/session)</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Carryover</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ZOOM (from Gurbachan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Prepare demo of business directory backend + data ingestion process for next Tuesday meeting</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>Due Tue</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>Work with Amira on documenting the search/scraping pipeline for the AI Business Directory</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Dev 2 — Samarveer Toor (Content &amp; NLP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NEW (from Guide/WBS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>WBS 2.1</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>Technical SEO Executor: Build auto-fix for sitemap.xml generation from scan results</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLEANUP (carryover)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Verify content-briefs and content-score endpoints work with DynamoDB (db_dynamo.py fallback)</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Carryover</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Merge dev2-samar-merge branch to main if not already done</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Carryover</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ZOOM (from Gurbachan)</t>
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>Send Gurbachan the OpenClaw research document for review</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>Research NVIDIA OpenShell for security layer before OpenClaw — implement if feasible</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Research two-way email send/receive solutions (SES vs ImprovMX vs iCloud) — report findings by Tuesday</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Due Tue</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>Provide iCloud email settings to Gurbachan for official business email setup</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Due Tue</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr"/>
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>Prepare demo of DynamoDB migration + OpenClaw agent for next meeting</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>Send Gurbachan the automation hub / content generation demo link for review</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>ASAP</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="inlineStr"/>
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>Dev 4 — Tabasum (Integrations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>GEO Executor: Implement FAQ schema auto-generation from scan results for social content (WBS 2.2)</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Dev 3 — Troy Sauriol (Data &amp; Infrastructure)</t>
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>Merge dev4-tabasum-integrations branch to main (18 tests passing, CRUD complete — overdue)</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NEW (from Guide/WBS)</t>
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>Resolve Facebook/Instagram account verification — use personal accounts per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>Set up official business accounts using personal accounts (not "business accounts") per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>WBS 6.2</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="inlineStr">
-        <is>
-          <t>Developer API: Document all 45+ API endpoints with request/response examples for team reference</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="inlineStr"/>
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>Work with Samarveer on email solution for social media account verification</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLEANUP (carryover)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>Prepare demo of social scheduler + publishing pipeline for next meeting</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="inlineStr">
-        <is>
-          <t>DynamoDB migration complete — monitor for any endpoint errors post-deploy</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>Monitoring</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr"/>
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>Dev 5 — Amira (Frontend &amp; UX)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>OpenClaw Gateway installed — wire up Phase 1 integration (report delivery via /hooks/agent)</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="inlineStr"/>
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="inlineStr">
+        <is>
+          <t>Basic Dashboard: Add before/after scan comparison view to audit results page (WBS 2.3)</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ZOOM (from Gurbachan)</t>
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>Wire PDF email gate to POST /api/collect-email endpoint (now live on Lambda with DynamoDB)</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C39" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>Fix admin dashboard role check — DynamoDB auth is deployed, test admin access with amira.robleh@gmail.com</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="inlineStr">
-        <is>
-          <t>Send Gurbachan the OpenClaw research document for review</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>ASAP</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr"/>
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>Investigate and document business directory data ingestion with Deepthi — prepare for Tuesday demo</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>Research NVIDIA OpenShell for security layer before OpenClaw — implement if feasible</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>This Week</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr"/>
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>Continue AI Business Directory frontend pages (category, compare, listing)</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B42" s="15" t="inlineStr">
-        <is>
-          <t>Prepare demo of DynamoDB migration + OpenClaw agent for next meeting</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>Due Tue</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="12" t="inlineStr">
-        <is>
-          <t>Dev 4 — Tabasum (Social &amp; Integrations)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NEW (from Guide/WBS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D46" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="15" t="inlineStr">
-        <is>
-          <t>WBS 2.2</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="inlineStr">
-        <is>
-          <t>GEO Executor: Implement FAQ schema auto-generation from scan results for social content</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="D47" s="15" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLEANUP (carryover)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B49" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C49" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D49" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>Merge dev4-tabasum-integrations branch to main (18 tests passing, CRUD complete)</t>
-        </is>
-      </c>
-      <c r="C50" s="15" t="inlineStr">
-        <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="D50" s="15" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>Resolve Facebook/Instagram account verification — use personal accounts per Gurbachan</t>
-        </is>
-      </c>
-      <c r="C51" s="15" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="D51" s="15" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ZOOM (from Gurbachan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B53" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C53" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B54" s="15" t="inlineStr">
-        <is>
-          <t>Set up official business accounts using personal accounts (not "business accounts") per Gurbachan</t>
-        </is>
-      </c>
-      <c r="C54" s="15" t="inlineStr">
-        <is>
-          <t>This Week</t>
-        </is>
-      </c>
-      <c r="D54" s="15" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B55" s="15" t="inlineStr">
-        <is>
-          <t>Work with Samarveer on email solution for social media account verification</t>
-        </is>
-      </c>
-      <c r="C55" s="15" t="inlineStr">
-        <is>
-          <t>This Week</t>
-        </is>
-      </c>
-      <c r="D55" s="15" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B56" s="15" t="inlineStr">
-        <is>
-          <t>Prepare demo of social scheduler + publishing pipeline for next meeting</t>
-        </is>
-      </c>
-      <c r="C56" s="15" t="inlineStr">
-        <is>
-          <t>Due Tue</t>
-        </is>
-      </c>
-      <c r="D56" s="15" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="12" t="inlineStr">
-        <is>
-          <t>Dev 5 — Amira Robleh (Frontend &amp; UX)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NEW (from Guide/WBS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C60" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D60" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t>WBS 2.3</t>
-        </is>
-      </c>
-      <c r="B61" s="15" t="inlineStr">
-        <is>
-          <t>Basic Dashboard: Add before/after scan comparison view to audit results page</t>
-        </is>
-      </c>
-      <c r="C61" s="15" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLEANUP (carryover)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B63" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C63" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B64" s="15" t="inlineStr">
-        <is>
-          <t>Wire PDF email gate to POST /api/collect-email endpoint (now live on Lambda)</t>
-        </is>
-      </c>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B65" s="15" t="inlineStr">
-        <is>
-          <t>Fix admin dashboard role check — DynamoDB auth is deployed, test admin access</t>
-        </is>
-      </c>
-      <c r="C65" s="15" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
-      <c r="D65" s="15" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ZOOM (from Gurbachan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C67" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D67" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B68" s="15" t="inlineStr">
-        <is>
-          <t>Investigate and document business directory data ingestion with Deepthi — prepare for Tuesday demo</t>
-        </is>
-      </c>
-      <c r="C68" s="15" t="inlineStr">
-        <is>
-          <t>Due Tue</t>
-        </is>
-      </c>
-      <c r="D68" s="15" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B69" s="15" t="inlineStr">
-        <is>
-          <t>Continue AI Business Directory frontend pages (category, compare, listing)</t>
-        </is>
-      </c>
-      <c r="C69" s="15" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B70" s="15" t="inlineStr">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="21" t="inlineStr">
         <is>
           <t>Set up proper business email infrastructure with SES (send + receive) per Gurbachan</t>
         </is>
       </c>
-      <c r="C70" s="15" t="inlineStr">
-        <is>
-          <t>This Week</t>
-        </is>
-      </c>
-      <c r="D70" s="15" t="inlineStr"/>
+      <c r="D42" s="21" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A17:D17"/>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A62:D62"/>
     <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Week Apr15-Apr22 tasks: 30 tasks, H100/H200 research, investor link, templates
</commit_message>
<xml_diff>
--- a/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
+++ b/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Mar26-Apr1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr1-Apr8" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr8-Apr15" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr15-Apr22" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,33 +57,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="16"/>
     </font>
@@ -99,7 +73,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -138,30 +112,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
-        <bgColor rgb="002F5496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C65911"/>
-        <bgColor rgb="00C65911"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007030A0"/>
-        <bgColor rgb="007030A0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="001A103C"/>
         <bgColor rgb="001A103C"/>
       </patternFill>
@@ -191,7 +141,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -214,27 +164,30 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -245,27 +198,17 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,1020 +575,1020 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
-    <col width="12" customWidth="1" style="9" min="1" max="2"/>
-    <col width="70" customWidth="1" style="9" min="3" max="3"/>
-    <col width="12" customWidth="1" style="9" min="4" max="4"/>
+    <col width="12" customWidth="1" style="7" min="1" max="2"/>
+    <col width="70" customWidth="1" style="7" min="3" max="3"/>
+    <col width="12" customWidth="1" style="7" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="9">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="21" customHeight="1" s="7">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>AI 1st SEO — Weekly Tasks (March 26 - April 1, 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="9">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4" ht="18" customHeight="1" s="7">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="27.6" customHeight="1" s="9">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="5" ht="27.6" customHeight="1" s="7">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Begin building GEO Scanner Agent — orchestrator skeleton that coordinates scanner agents and returns structured results</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="27.6" customHeight="1" s="9">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27.6" customHeight="1" s="7">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Wire GEO probe results to RDS — call POST /api/data/geo-probes and POST /api/data/ai-visibility from GEO engine</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Continue improving scanner output for non-technical users (Gurbachan feedback)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Build comprehensive parameter reference list for AI visibility scanning</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Add URL/link to new GEO page in admin dashboard, send to Gurbachan for review</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="27.6" customHeight="1" s="9">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="27.6" customHeight="1" s="7">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Document and diagram SEO and content analysis workflows (process + value-add steps)</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Deploy microproject to Linux server using OpenShell/NVIDIA open shell layer</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Share deployment instructions with team</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="9">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="7">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="27.6" customHeight="1" s="9">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="15" ht="27.6" customHeight="1" s="7">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Build content scoring engine — expand compute_readability_score, compute_seo_score, compute_aeo_score to full 13+13 checks per DEV2-CHANGES.md</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="27.6" customHeight="1" s="9">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="27.6" customHeight="1" s="7">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Add get_content_briefs() and get_content_brief_by_id() to db.py — /api/content-briefs returns 500 without them</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Fix merge conflicts from this week's deploys</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="27.6" customHeight="1" s="9">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="27.6" customHeight="1" s="7">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Ensure Ollama fallback chain works end-to-end (Nova Lite → Ollama sageaios → Ollama databi → raw SERP)</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Fix content brief generation and AI recommendations</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Deploy microproject to Linux server</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Share deployment instructions with team</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1" s="9">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="7">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="27.6" customHeight="1" s="9">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="24" ht="27.6" customHeight="1" s="7">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Build api_request_log middleware for tracking API usage — feeds admin dashboard analytics and future billing</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="27.6" customHeight="1" s="9">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="27.6" customHeight="1" s="7">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Fully terminate EC2 and delete all associated resources (Elastic IPs, security groups, snapshots)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Coordinate with Amira on admin dashboard API if she needs changes</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="27.6" customHeight="1" s="9">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="27.6" customHeight="1" s="7">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Verify all EC2-related resources fully deleted (IPs, databases, sub-services) — Gurbachan stressed this</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Compile and send AI notes + task updates to team via WhatsApp</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Deploy microproject to Linux server</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Share deployment instructions with team</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="27.6" customHeight="1" s="9">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="27.6" customHeight="1" s="7">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Note: Main website updates (About Us, Privacy, Contact) = Amira's responsibility. Troy provides backend support if needed.</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1" s="9">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="7">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Dev 4 — Tabasum (Integrations)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="27.6" customHeight="1" s="9">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="34" ht="27.6" customHeight="1" s="7">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Build social media content generation pipeline — use SEO info document as input for AI-generated posts via LLM fallback chain</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Complete social post scheduler CRUD — data API at /api/data/social-posts is ready</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Follow up with Gurbachan on Facebook/LinkedIn business account linking</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Test auth with direct Gmail address (not @ai1stseo.com forwarded)</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Implement Facebook and LinkedIn scheduling per Gurbachan's instructions</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Collect and store SEO info (Google, AEO, GEO) into document for AI content generation</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Test and potentially integrate PostIZ for social media scheduling on AWS</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Email Paul and Gurbachan re: DynamoDB permission issues for Lambda execution role</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Troubleshoot forgot password email functionality</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Deploy microproject to Linux server</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Share deployment instructions with team</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1" s="9">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="7">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>Dev 5 — Amira (Frontend &amp; UX)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="27.6" customHeight="1" s="9">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="47" ht="27.6" customHeight="1" s="7">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Build admin dashboard UI using Troy's API endpoints — see AMIRA_ADMIN_HANDOFF.md and admin.html reference</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Separate user dashboard from admin dashboard (ongoing from Mar 24)</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Continue React + Vite migration</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Coordinate with Samarveer on S3 deploys to avoid overwrites</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="27.6" customHeight="1" s="9">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="27.6" customHeight="1" s="7">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Move non-essential resources/diagrams/buttons from main website to admin dashboard</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="27.6" customHeight="1" s="9">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="27.6" customHeight="1" s="7">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Update main website: professional, advertising-friendly (About Us, Privacy Policy, Contact, developer info)</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Add free analysis section with PDF report feature (for marketing)</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Deploy microproject to Linux server</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Share deployment instructions with team</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1669,976 +1612,976 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
-    <col width="12" customWidth="1" style="9" min="1" max="2"/>
-    <col width="70" customWidth="1" style="9" min="3" max="3"/>
-    <col width="12" customWidth="1" style="9" min="4" max="4"/>
+    <col width="12" customWidth="1" style="7" min="1" max="2"/>
+    <col width="70" customWidth="1" style="7" min="3" max="3"/>
+    <col width="12" customWidth="1" style="7" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="9">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="21" customHeight="1" s="7">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>AI 1st SEO — Weekly Tasks (April 1 - April 8, 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="9">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4" ht="18" customHeight="1" s="7">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="27.6" customHeight="1" s="9">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="5" ht="27.6" customHeight="1" s="7">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Conduct R&amp;D on Agent Core functionality (from guide Phase 1 — orchestrator + scanner agents)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="27.6" customHeight="1" s="9">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27.6" customHeight="1" s="7">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Review AI Business Directory document from Gurbachan and begin database setup on his server</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Continue Month 1 Research deliverables (8 API endpoints + UI — in progress)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Ensure GEO scanner agent works end-to-end on her own Lambda (ai1stseo-geo-engine)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Work with Amira on overlapping SEO audit work and AI Business Directory project</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Show progress on AI Business Directory understanding/setup by next meeting</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Test Nova Lite for multi-modal content creation (images, videos) and report capabilities</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="9">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="7">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Migrate content briefs persistence from RDS to DynamoDB per Gurbachan's directive</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Build content scoring engine with full 13+13 checks (carryover — still needed)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="27.6" customHeight="1" s="9">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="27.6" customHeight="1" s="7">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Add get_content_briefs() and get_content_brief_by_id() to db.py (still missing from last week)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Ensure Ollama fallback chain works end-to-end</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Fix any remaining merge conflicts</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Extract necessary data from RDS before Troy shuts it down</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Test Nova Lite for multi-modal content creation and report capabilities</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1" s="9">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="7">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="27.6" customHeight="1" s="9">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="23" ht="27.6" customHeight="1" s="7">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Begin working with OpenClaw on Gurbachan's server and report on integration progress</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="27.6" customHeight="1" s="9">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="27.6" customHeight="1" s="7">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Plan DynamoDB migration strategy — map existing RDS tables to DynamoDB table designs per Gurbachan's directive</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Verify EC2 fully terminated and no lingering resources (done — confirm with Paul)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Coordinate with team on RDS data extraction before shutdown</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Shut down Lightsail service to prevent further costs (ensure no data loss)</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Done (Amira)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="27.6" customHeight="1" s="9">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="28" ht="27.6" customHeight="1" s="7">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Shut down RDS/Postgres after confirming all team members have extracted necessary data</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Update and share current week's tasks in Excel spreadsheet via WhatsApp</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="27.6" customHeight="1" s="9">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="27.6" customHeight="1" s="7">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Note: Gurbachan is moving away from Postgres to individual DynamoDB tables per app. Plan migration accordingly.</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1" s="9">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="7">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Dev 4 — Tabasum (Integrations)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="27.6" customHeight="1" s="9">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="33" ht="27.6" customHeight="1" s="7">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Build multi-modal content pipeline — test Nova Lite and Ollama for image/video generation</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Explore Reddit integration for social media posting</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Continue resolving social media API connection issues (Facebook, Instagram, LinkedIn)</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done  </t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Ensure marketing@ email can both send and receive replies for automation</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done  </t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Complete social post scheduler CRUD (PR still unmerged — push to main)</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done  </t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Work with Samarveer (Summer) to resolve social media API connection issues</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Test TikTok video posting and evaluate usefulness</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Show progress/achievements on social media pipeline by next meeting</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done  </t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Deposit $5 into account for social media posting (per Gurbachan)</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Test Nova Lite for multi-modal content creation (images, videos)</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1" s="9">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="44" ht="18" customHeight="1" s="7">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t>Dev 5 — Amira (Frontend &amp; UX)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Build email gate on PDF audit download — collect email before allowing download</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Begin AI Business Directory project setup with Deepthi</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="27.6" customHeight="1" s="9">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="27.6" customHeight="1" s="7">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Continue main website updates (About Us, Privacy Policy, Contact — contact.html is ready on repo)</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Deploy contact.html to Amplify and link from homepage footer</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Share admin dashboard passwords with team or help them create accounts</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Work with Deepthi on overlapping SEO audit work and AI Business Directory</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Review AI Business Directory document from Gurbachan</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Show progress on AI Business Directory understanding/setup by next meeting</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Forward AI notes to team for review</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2662,18 +2605,770 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
+  <cols>
+    <col width="12" customWidth="1" style="7" min="1" max="1"/>
+    <col width="13" customWidth="1" style="7" min="2" max="2"/>
+    <col width="90.28515625" customWidth="1" style="7" min="3" max="3"/>
+    <col width="12" customWidth="1" style="7" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1" s="7">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>AI 1st SEO — Weekly Tasks (April 8 - April 15, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="7">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Dev 1 — Deepthi (AI/ML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>GEO Scanner: Add 5 new AI-readiness criteria to probe engine (WBS 1.3 — target 25 total GEO criteria)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Investigate and document how business directory data is ingested into DynamoDB — prepare backend walkthrough for next meeting</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Ensure all GEO routes work on Lambda after DynamoDB migration (test geo-probe/models, aeo/analyze, chatbot/session)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Prepare demo of business directory backend + data ingestion process for next Tuesday meeting</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Work with Amira on documenting the search/scraping pipeline for the AI Business Directory</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Prepare to present backend details and search process at next meeting</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="7">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Technical SEO Executor: Build auto-fix for sitemap.xml generation from scan results (WBS 2.1)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Verify content-briefs and content-score endpoints work with DynamoDB (db_dynamo.py fallback)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Merge dev2-samar-merge branch to main if not already done</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Research two-way email send/receive solutions (SES vs ImprovMX vs iCloud) — report findings by Tuesday</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Provide iCloud email settings to Gurbachan for official business email setup</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Send Gurbachan the automation hub / content generation demo link for review</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="7">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Developer API: Document all 45+ API endpoints with request/response examples for team reference (WBS 6.2)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>DynamoDB migration complete — monitor for any endpoint errors post-deploy</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>OpenClaw Gateway installed — wire up Phase 1 integration (report delivery via /hooks/agent)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Send Gurbachan the OpenClaw research document for review</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Research NVIDIA OpenShell for security layer before OpenClaw — implement if feasible</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Prepare demo of DynamoDB migration + OpenClaw agent for next meeting</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="7">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Dev 4 — Tabasum (Integrations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>GEO Executor: Implement FAQ schema auto-generation from scan results for social content (WBS 2.2)</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Merge dev4-tabasum-integrations branch to main (18 tests passing, CRUD complete — overdue)</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Resolve Facebook/Instagram account verification — use personal accounts per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Set up official business accounts using personal accounts (not "business accounts") per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Work with Samarveer on email solution for social media account verification</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Prepare demo of social scheduler + publishing pipeline for next meeting</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="7">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Dev 5 — Amira (Frontend &amp; UX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Basic Dashboard: Add before/after scan comparison view to audit results page (WBS 2.3)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Wire PDF email gate to POST /api/collect-email endpoint (now live on Lambda with DynamoDB)</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Fix admin dashboard role check — DynamoDB auth is deployed, test admin access with amira.robleh@gmail.com</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Investigate and document business directory data ingestion with Deepthi — prepare for Tuesday demo</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Continue AI Business Directory frontend pages (category, compare, listing)</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Set up proper business email infrastructure with SES (send + receive) per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A36:D36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="9" min="1" max="1"/>
-    <col width="13" customWidth="1" style="9" min="2" max="2"/>
-    <col width="70" customWidth="1" style="9" min="3" max="3"/>
-    <col width="12" customWidth="1" style="9" min="4" max="4"/>
+    <col width="12" customWidth="1" style="7" min="1" max="1"/>
+    <col width="13" customWidth="1" style="7" min="2" max="2"/>
+    <col width="70" customWidth="1" style="7" min="3" max="3"/>
+    <col width="12" customWidth="1" style="7" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>AI 1st SEO — Weekly Tasks (April 8 - April 15, 2026)</t>
+          <t>AI 1st SEO — Weekly Tasks (April 15 - April 22, 2026)</t>
         </is>
       </c>
     </row>
@@ -2707,132 +3402,132 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>GEO Scanner: Add 5 new AI-readiness criteria to probe engine (WBS 1.3 — target 25 total GEO criteria)</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>GEO Scanner: Expand AI-readiness criteria to 25 total and validate against live sites (WBS 1.3 continued)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>Investigate and document how business directory data is ingested into DynamoDB — prepare backend walkthrough for next meeting</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Provide estimate of records being added to directory database daily — present at next meeting</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>Ensure all GEO routes work on Lambda after DynamoDB migration (test geo-probe/models, aeo/analyze, chatbot/session)</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Continue data scraping pipeline for Ottawa business records — ensure scraper runs continuously</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>Prepare demo of business directory backend + data ingestion process for next Tuesday meeting</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>Work with Amira on documenting the search/scraping pipeline for the AI Business Directory</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Collaborate with Amira, Tabasum, Samarveer on accelerator usage plan and recommendations for Gurbachan</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>Prepare to present backend details and search process at next meeting</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -2846,132 +3541,132 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>Technical SEO Executor: Build auto-fix for sitemap.xml generation from scan results (WBS 2.1)</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Technical SEO Executor: Build auto-fix for robots.txt generation from scan results (WBS 2.1 continued)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>Verify content-briefs and content-score endpoints work with DynamoDB (db_dynamo.py fallback)</t>
-        </is>
-      </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Develop 3-4 perfect AEO/GEO/SEO templates for different business types (service, manufacturing, etc.) — per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C15" s="21" t="inlineStr">
-        <is>
-          <t>Merge dev2-samar-merge branch to main if not already done</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Determine how many possible template types are needed and document the scoring benchmarks (100% target)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>Research two-way email send/receive solutions (SES vs ImprovMX vs iCloud) — report findings by Tuesday</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Ensure keyword clustering tool is stable on main after the app.py overwrite fix</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>Provide iCloud email settings to Gurbachan for official business email setup</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate how they could improve keyword analysis and NLP work</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>Send Gurbachan the automation hub / content generation demo link for review</t>
-        </is>
-      </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -2985,132 +3680,132 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B21" s="22" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>Developer API: Document all 45+ API endpoints with request/response examples for team reference (WBS 6.2)</t>
-        </is>
-      </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Developer API: Add rate limiting dashboard and usage analytics per API key (WBS 6.2 continued)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C22" s="21" t="inlineStr">
-        <is>
-          <t>DynamoDB migration complete — monitor for any endpoint errors post-deploy</t>
-        </is>
-      </c>
-      <c r="D22" s="21" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Add "investor" contact option/link at the bottom of the homepage for potential investors</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>OpenClaw Gateway installed — wire up Phase 1 integration (report delivery via /hooks/agent)</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Send final email to Gurbachan (CC Paul) re: OpenClaw/OpenShell Podman UDP socket permission issue</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>Send Gurbachan the OpenClaw research document for review</t>
-        </is>
-      </c>
-      <c r="D24" s="21" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>OpenShell sandbox — blocked on LXC seccomp restriction, waiting on Gurbachan</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>Research NVIDIA OpenShell for security layer before OpenClaw — implement if feasible</t>
-        </is>
-      </c>
-      <c r="D25" s="21" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 accelerator pricing and develop a usage plan for the team’s tiered job system</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>Prepare demo of DynamoDB migration + OpenClaw agent for next meeting</t>
-        </is>
-      </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -3124,132 +3819,132 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B29" s="22" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>GEO Executor: Implement FAQ schema auto-generation from scan results for social content (WBS 2.2)</t>
-        </is>
-      </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>GEO Executor: Implement Q&amp;A markup auto-generation from scan results for social content (WBS 2.2 continued)</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B30" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>Merge dev4-tabasum-integrations branch to main (18 tests passing, CRUD complete — overdue)</t>
-        </is>
-      </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Modify website email capture prompt — emphasize "free analysis" instead of "starter kit", list AEO/GEO before SEO</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>Resolve Facebook/Instagram account verification — use personal accounts per Gurbachan</t>
-        </is>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Send Paul email requesting SES SMTP permissions and additional credentials for marketing email</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B32" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>Set up official business accounts using personal accounts (not "business accounts") per Gurbachan</t>
-        </is>
-      </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B33" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>Work with Samarveer on email solution for social media account verification</t>
-        </is>
-      </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Collaborate with Deepthi, Amira, Samarveer on accelerator usage plan and recommendations for Gurbachan</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B34" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C34" s="21" t="inlineStr">
-        <is>
-          <t>Prepare demo of social scheduler + publishing pipeline for next meeting</t>
-        </is>
-      </c>
-      <c r="D34" s="21" t="inlineStr">
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -3263,132 +3958,132 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C37" s="21" t="inlineStr">
-        <is>
-          <t>Basic Dashboard: Add before/after scan comparison view to audit results page (WBS 2.3)</t>
-        </is>
-      </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Basic Dashboard: Add score trend chart showing historical audit scores over time (WBS 2.3 continued)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B38" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>Wire PDF email gate to POST /api/collect-email endpoint (now live on Lambda with DynamoDB)</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="inlineStr">
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Update before/after scan comparison tool — display highest changes at the top per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B39" s="23" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>Fix admin dashboard role check — DynamoDB auth is deployed, test admin access with amira.robleh@gmail.com</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Wire Documents tab to live API endpoints (backend is deployed and matching your schema)</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B40" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>Investigate and document business directory data ingestion with Deepthi — prepare for Tuesday demo</t>
-        </is>
-      </c>
-      <c r="D40" s="21" t="inlineStr">
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Wire PDF email gate to POST /api/collect-email endpoint (live on Lambda)</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B41" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>Continue AI Business Directory frontend pages (category, compare, listing)</t>
-        </is>
-      </c>
-      <c r="D41" s="21" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B42" s="24" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>Set up proper business email infrastructure with SES (send + receive) per Gurbachan</t>
-        </is>
-      </c>
-      <c r="D42" s="21" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>

</xml_diff>

<commit_message>
Fix Week Apr15-Apr22: align Dev 2 (content templates) and Dev 4 (social API integration) tasks to proper roles
</commit_message>
<xml_diff>
--- a/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
+++ b/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
@@ -3372,6 +3372,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -3533,6 +3534,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
@@ -3553,7 +3555,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Technical SEO Executor: Build auto-fix for robots.txt generation from scan results (WBS 2.1 continued)</t>
+          <t>Content scoring engine: Build AEO/GEO/SEO benchmark templates for service and manufacturing business types (WBS 4.1 — content criteria)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -3672,6 +3674,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
@@ -3811,6 +3814,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
@@ -3831,7 +3835,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>GEO Executor: Implement Q&amp;A markup auto-generation from scan results for social content (WBS 2.2 continued)</t>
+          <t>Social media API integration: Connect Buffer/Postiz publishers to live platform accounts and test end-to-end posting (WBS 3.4 — platform adapter)</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -3950,6 +3954,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Week Apr22-Apr29 tasks: 30 tasks, Invest Ottawa demo prep, H100 experiments, content freshness
</commit_message>
<xml_diff>
--- a/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
+++ b/OneDrive/Desktop/seo deployment/WEEKLY_TASKS.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="2" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Mar26-Apr1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr1-Apr8" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr8-Apr15" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr15-Apr22" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week Apr22-Apr29" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -168,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,17 +178,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -198,11 +197,40 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -575,56 +603,56 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="12" customWidth="1" style="7" min="1" max="2"/>
-    <col width="70" customWidth="1" style="7" min="3" max="3"/>
-    <col width="12" customWidth="1" style="7" min="4" max="4"/>
+    <col width="12" customWidth="1" style="23" min="1" max="2"/>
+    <col width="70" customWidth="1" style="23" min="3" max="3"/>
+    <col width="12" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="7">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="21" customHeight="1" s="23">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>AI 1st SEO — Weekly Tasks (March 26 - April 1, 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="7">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="4" ht="18" customHeight="1" s="23">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="27.6" customHeight="1" s="7">
+    <row r="5" ht="27.6" customHeight="1" s="23">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -640,13 +668,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="27.6" customHeight="1" s="7">
+    <row r="6" ht="27.6" customHeight="1" s="23">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -668,7 +696,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -690,7 +718,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -712,7 +740,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -728,13 +756,13 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="27.6" customHeight="1" s="7">
+    <row r="10" ht="27.6" customHeight="1" s="23">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -756,7 +784,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -778,7 +806,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -794,20 +822,20 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="7">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="14" ht="18" customHeight="1" s="23">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="27.6" customHeight="1" s="7">
+    <row r="15" ht="27.6" customHeight="1" s="23">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -823,13 +851,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="27.6" customHeight="1" s="7">
+    <row r="16" ht="27.6" customHeight="1" s="23">
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -851,7 +879,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -867,13 +895,13 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="27.6" customHeight="1" s="7">
+    <row r="18" ht="27.6" customHeight="1" s="23">
       <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -895,7 +923,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -917,7 +945,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -939,7 +967,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -955,20 +983,20 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1" s="7">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="23" ht="18" customHeight="1" s="23">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="27.6" customHeight="1" s="7">
+    <row r="24" ht="27.6" customHeight="1" s="23">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -984,13 +1012,13 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="27.6" customHeight="1" s="7">
+    <row r="25" ht="27.6" customHeight="1" s="23">
       <c r="A25" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1012,7 +1040,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1028,13 +1056,13 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="27.6" customHeight="1" s="7">
+    <row r="27" ht="27.6" customHeight="1" s="23">
       <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1056,7 +1084,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1078,7 +1106,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1100,7 +1128,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1116,13 +1144,13 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="27.6" customHeight="1" s="7">
+    <row r="31" ht="27.6" customHeight="1" s="23">
       <c r="A31" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1138,20 +1166,20 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1" s="7">
-      <c r="A33" s="9" t="inlineStr">
+    <row r="33" ht="18" customHeight="1" s="23">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>Dev 4 — Tabasum (Integrations)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="27.6" customHeight="1" s="7">
+    <row r="34" ht="27.6" customHeight="1" s="23">
       <c r="A34" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1173,7 +1201,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1195,7 +1223,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1217,7 +1245,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1239,7 +1267,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1261,7 +1289,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1283,7 +1311,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1305,7 +1333,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1327,7 +1355,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1349,7 +1377,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1371,7 +1399,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1387,20 +1415,20 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1" s="7">
-      <c r="A46" s="9" t="inlineStr">
+    <row r="46" ht="18" customHeight="1" s="23">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t>Dev 5 — Amira (Frontend &amp; UX)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="27.6" customHeight="1" s="7">
+    <row r="47" ht="27.6" customHeight="1" s="23">
       <c r="A47" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B47" s="10" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1422,7 +1450,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1444,7 +1472,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1466,7 +1494,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1482,13 +1510,13 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="27.6" customHeight="1" s="7">
+    <row r="51" ht="27.6" customHeight="1" s="23">
       <c r="A51" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1504,13 +1532,13 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="27.6" customHeight="1" s="7">
+    <row r="52" ht="27.6" customHeight="1" s="23">
       <c r="A52" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1532,7 +1560,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1554,7 +1582,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1576,7 +1604,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1612,56 +1640,56 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="12" customWidth="1" style="7" min="1" max="2"/>
-    <col width="70" customWidth="1" style="7" min="3" max="3"/>
-    <col width="12" customWidth="1" style="7" min="4" max="4"/>
+    <col width="12" customWidth="1" style="23" min="1" max="2"/>
+    <col width="70" customWidth="1" style="23" min="3" max="3"/>
+    <col width="12" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="7">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="21" customHeight="1" s="23">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>AI 1st SEO — Weekly Tasks (April 1 - April 8, 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="7">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="4" ht="18" customHeight="1" s="23">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="27.6" customHeight="1" s="7">
+    <row r="5" ht="27.6" customHeight="1" s="23">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1673,17 +1701,17 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="27.6" customHeight="1" s="7">
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27.6" customHeight="1" s="23">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1695,7 +1723,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
@@ -1705,7 +1733,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1717,7 +1745,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
@@ -1727,7 +1755,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1739,7 +1767,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
@@ -1749,7 +1777,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1761,7 +1789,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
@@ -1771,7 +1799,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1783,7 +1811,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
@@ -1793,7 +1821,7 @@
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1805,12 +1833,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="7">
-      <c r="A13" s="9" t="inlineStr">
+          <t xml:space="preserve">done </t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="23">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
         </is>
@@ -1822,7 +1850,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1844,7 +1872,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1860,13 +1888,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="27.6" customHeight="1" s="7">
+    <row r="16" ht="27.6" customHeight="1" s="23">
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1888,7 +1916,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1910,7 +1938,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -1932,7 +1960,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1954,7 +1982,7 @@
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -1970,20 +1998,20 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" s="7">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="22" ht="18" customHeight="1" s="23">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="27.6" customHeight="1" s="7">
+    <row r="23" ht="27.6" customHeight="1" s="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -1999,13 +2027,13 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="27.6" customHeight="1" s="7">
+    <row r="24" ht="27.6" customHeight="1" s="23">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -2027,7 +2055,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2049,7 +2077,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2071,7 +2099,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2087,13 +2115,13 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="27.6" customHeight="1" s="7">
+    <row r="28" ht="27.6" customHeight="1" s="23">
       <c r="A28" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2115,7 +2143,7 @@
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2131,13 +2159,13 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="27.6" customHeight="1" s="7">
+    <row r="30" ht="27.6" customHeight="1" s="23">
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2153,20 +2181,20 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1" s="7">
-      <c r="A32" s="9" t="inlineStr">
+    <row r="32" ht="18" customHeight="1" s="23">
+      <c r="A32" s="24" t="inlineStr">
         <is>
           <t>Dev 4 — Tabasum (Integrations)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="27.6" customHeight="1" s="7">
+    <row r="33" ht="27.6" customHeight="1" s="23">
       <c r="A33" s="1" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -2188,7 +2216,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -2210,7 +2238,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2232,7 +2260,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2254,7 +2282,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2276,7 +2304,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2298,7 +2326,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2320,7 +2348,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2342,7 +2370,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2364,7 +2392,7 @@
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2380,8 +2408,8 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1" s="7">
-      <c r="A44" s="9" t="inlineStr">
+    <row r="44" ht="18" customHeight="1" s="23">
+      <c r="A44" s="24" t="inlineStr">
         <is>
           <t>Dev 5 — Amira (Frontend &amp; UX)</t>
         </is>
@@ -2393,7 +2421,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -2415,7 +2443,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -2431,13 +2459,13 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="27.6" customHeight="1" s="7">
+    <row r="47" ht="27.6" customHeight="1" s="23">
       <c r="A47" s="1" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2459,7 +2487,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2481,7 +2509,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
@@ -2503,7 +2531,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2525,7 +2553,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2547,7 +2575,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2569,7 +2597,7 @@
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>Zoom</t>
         </is>
@@ -2605,733 +2633,733 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="12" customWidth="1" style="7" min="1" max="1"/>
-    <col width="13" customWidth="1" style="7" min="2" max="2"/>
-    <col width="90.28515625" customWidth="1" style="7" min="3" max="3"/>
-    <col width="12" customWidth="1" style="7" min="4" max="4"/>
+    <col width="12" customWidth="1" style="23" min="1" max="1"/>
+    <col width="13" customWidth="1" style="23" min="2" max="2"/>
+    <col width="90.33203125" customWidth="1" style="23" min="3" max="3"/>
+    <col width="12" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="7">
-      <c r="A1" s="13" t="inlineStr">
+    <row r="1" ht="21" customHeight="1" s="23">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>AI 1st SEO — Weekly Tasks (April 8 - April 15, 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="7">
-      <c r="A4" s="14" t="inlineStr">
+    <row r="4" ht="18" customHeight="1" s="23">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>GEO Scanner: Add 5 new AI-readiness criteria to probe engine (WBS 1.3 — target 25 total GEO criteria)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Investigate and document how business directory data is ingested into DynamoDB — prepare backend walkthrough for next meeting</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Ensure all GEO routes work on Lambda after DynamoDB migration (test geo-probe/models, aeo/analyze, chatbot/session)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Prepare demo of business directory backend + data ingestion process for next Tuesday meeting</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Work with Amira on documenting the search/scraping pipeline for the AI Business Directory</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">done </t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Prepare to present backend details and search process at next meeting</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="7">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">done </t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="23">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Technical SEO Executor: Build auto-fix for sitemap.xml generation from scan results (WBS 2.1)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Verify content-briefs and content-score endpoints work with DynamoDB (db_dynamo.py fallback)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Merge dev2-samar-merge branch to main if not already done</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Research two-way email send/receive solutions (SES vs ImprovMX vs iCloud) — report findings by Tuesday</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Provide iCloud email settings to Gurbachan for official business email setup</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Send Gurbachan the automation hub / content generation demo link for review</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="7">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="23">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Developer API: Document all 45+ API endpoints with request/response examples for team reference (WBS 6.2)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>DynamoDB migration complete — monitor for any endpoint errors post-deploy</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>OpenClaw Gateway installed — wire up Phase 1 integration (report delivery via /hooks/agent)</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Send Gurbachan the OpenClaw research document for review</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Research NVIDIA OpenShell for security layer before OpenClaw — implement if feasible</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Prepare demo of DynamoDB migration + OpenClaw agent for next meeting</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1" s="7">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="23">
+      <c r="A28" s="25" t="inlineStr">
         <is>
           <t>Dev 4 — Tabasum (Integrations)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>GEO Executor: Implement FAQ schema auto-generation from scan results for social content (WBS 2.2)</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Merge dev4-tabasum-integrations branch to main (18 tests passing, CRUD complete — overdue)</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Resolve Facebook/Instagram account verification — use personal accounts per Gurbachan</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Set up official business accounts using personal accounts (not "business accounts") per Gurbachan</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Work with Samarveer on email solution for social media account verification</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Prepare demo of social scheduler + publishing pipeline for next meeting</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1" s="7">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="23">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>Dev 5 — Amira (Frontend &amp; UX)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B37" s="15" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Basic Dashboard: Add before/after scan comparison view to audit results page (WBS 2.3)</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Wire PDF email gate to POST /api/collect-email endpoint (now live on Lambda with DynamoDB)</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B39" s="16" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Fix admin dashboard role check — DynamoDB auth is deployed, test admin access with amira.robleh@gmail.com</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Investigate and document business directory data ingestion with Deepthi — prepare for Tuesday demo</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B41" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Continue AI Business Directory frontend pages (category, compare, listing)</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B42" s="17" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Set up proper business email infrastructure with SES (send + receive) per Gurbachan</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -3356,739 +3384,1527 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="12" customWidth="1" style="23" min="1" max="1"/>
+    <col width="13" customWidth="1" style="23" min="2" max="2"/>
+    <col width="74.109375" customWidth="1" style="23" min="3" max="3"/>
+    <col width="12" customWidth="1" style="23" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.6" customHeight="1" s="23">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>AI 1st SEO — Weekly Tasks (April 15 - April 22, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="n"/>
+      <c r="B2" s="20" t="n"/>
+      <c r="C2" s="20" t="n"/>
+      <c r="D2" s="20" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="23">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Dev 1 — Deepthi (AI/ML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="27.6" customHeight="1" s="23">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>GEO Scanner: Expand AI-readiness criteria to 25 total and validate against live sites (WBS 1.3 continued)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27.6" customHeight="1" s="23">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Provide estimate of records being added to directory database daily — present at next meeting</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="27.6" customHeight="1" s="23">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Continue data scraping pipeline for Ottawa business records — ensure scraper runs continuously</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="27.6" customHeight="1" s="23">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="27.6" customHeight="1" s="23">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Collaborate with Amira, Tabasum, Samarveer on accelerator usage plan and recommendations for Gurbachan</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="n"/>
+      <c r="B11" s="20" t="n"/>
+      <c r="C11" s="20" t="n"/>
+      <c r="D11" s="20" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="23">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="27.6" customHeight="1" s="23">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Content scoring engine: Build AEO/GEO/SEO benchmark templates for service and manufacturing business types (WBS 4.1 — content criteria)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="27.6" customHeight="1" s="23">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Develop 3-4 perfect AEO/GEO/SEO templates for different business types (service, manufacturing, etc.) — per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="27.6" customHeight="1" s="23">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Determine how many possible template types are needed and document the scoring benchmarks (100% target)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Ensure keyword clustering tool is stable on main after the app.py overwrite fix</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="27.6" customHeight="1" s="23">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate how they could improve keyword analysis and NLP work</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="n"/>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="23">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="27.6" customHeight="1" s="23">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Developer API: Add rate limiting dashboard and usage analytics per API key (WBS 6.2 continued)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Add "investor" contact option/link at the bottom of the homepage for potential investors</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="27.6" customHeight="1" s="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Send final email to Gurbachan (CC Paul) re: OpenClaw/OpenShell Podman UDP socket permission issue</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="110.4" customHeight="1" s="23">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>OpenShell sandbox — blocked on LXC seccomp restriction, waiting on Gurbachan</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Waiting on reply from Paul/Gurbachan with permissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="27.6" customHeight="1" s="23">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 accelerator pricing and develop a usage plan for the team’s tiered job system</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="n"/>
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="23">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Dev 4 — Tabasum (Integrations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="27.6" customHeight="1" s="23">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Social media API integration: Connect Buffer/Postiz publishers to live platform accounts and test end-to-end posting (WBS 3.4 — platform adapter)</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doing in steps based on the plan Mr Gurbachan sent me. </t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="27.6" customHeight="1" s="23">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Modify website email capture prompt — emphasize "free analysis" instead of "starter kit", list AEO/GEO before SEO</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="27.6" customHeight="1" s="23">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Send Paul email requesting SES SMTP permissions and additional credentials for marketing email</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="27.6" customHeight="1" s="23">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="27.6" customHeight="1" s="23">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Collaborate with Deepthi, Amira, Samarveer on accelerator usage plan and recommendations for Gurbachan</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20" t="n"/>
+      <c r="B35" s="20" t="n"/>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="23">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Dev 5 — Amira (Frontend &amp; UX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="27.6" customHeight="1" s="23">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Basic Dashboard: Add score trend chart showing historical audit scores over time (WBS 2.3 continued)</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="27.6" customHeight="1" s="23">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Update before/after scan comparison tool — display highest changes at the top per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Wire Documents tab to live API endpoints (backend is deployed and matching your schema)</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Wire PDF email gate to POST /api/collect-email endpoint (live on Lambda)</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="27.6" customHeight="1" s="23">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A36:D36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="7" min="1" max="1"/>
-    <col width="13" customWidth="1" style="7" min="2" max="2"/>
-    <col width="70" customWidth="1" style="7" min="3" max="3"/>
-    <col width="12" customWidth="1" style="7" min="4" max="4"/>
+    <col width="12" customWidth="1" style="23" min="1" max="1"/>
+    <col width="13" customWidth="1" style="23" min="2" max="2"/>
+    <col width="70" customWidth="1" style="23" min="3" max="3"/>
+    <col width="12" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>AI 1st SEO — Weekly Tasks (April 15 - April 22, 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>AI 1st SEO — Weekly Tasks (April 22 - April 29, 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Dev 1 — Deepthi (AI/ML)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>GEO Scanner: Expand AI-readiness criteria to 25 total and validate against live sites (WBS 1.3 continued)</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>GEO Scanner: Implement off-page SEO signal detection for backlink and domain authority analysis (WBS 4.3)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Provide estimate of records being added to directory database daily — present at next meeting</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Add benchmark brands and real multi-brand data flows to GEO Score Tracker and keyword performance register</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Continue data scraping pipeline for Ottawa business records — ensure scraper runs continuously</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Ensure directory page scraper runs continuously every 6 hours — monitor for crashes, extend timing per Gurbachan</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Research and implement tools for continuous daily content creation with time-stamped freshness (with Amira)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Collaborate with Amira, Tabasum, Samarveer on accelerator usage plan and recommendations for Gurbachan</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Conduct H100/H200 GPU experiments (4-5 hrs) — evaluate speed/quality for keyword analysis, present findings (with Amira)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Dev 1</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Prepare all tools and features for Invest Ottawa demo by third week of May</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Dev 2 — Samarveer (Content &amp; NLP)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Content scoring engine: Build AEO/GEO/SEO benchmark templates for service and manufacturing business types (WBS 4.1 — content criteria)</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Content Optimizer: Build LLM-powered content rewrite suggestions from audit results (WBS 5.1)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Dev 2</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Integrate template benchmark engine with Amira’s historical analysis / score tracking features</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Investigate where "AI First SEO" is mentioned or ranked in Claude, Gemini, and other AI platforms</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Explore multi-agent AI system where different agents assess and update website content for changing AI models</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Share competitor website examples with team for UI/UX inspiration</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Dev 2</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Prepare template benchmarks and content tools for Invest Ottawa demo by third week of May</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Develop 3-4 perfect AEO/GEO/SEO templates for different business types (service, manufacturing, etc.) — per Gurbachan</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Dev 2</t>
-        </is>
-      </c>
-      <c r="B15" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Determine how many possible template types are needed and document the scoring benchmarks (100% target)</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Dev 2</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Ensure keyword clustering tool is stable on main after the app.py overwrite fix</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Dev 2</t>
-        </is>
-      </c>
-      <c r="B17" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Research Amazon H100/H200 GPU accelerators — evaluate how they could improve keyword analysis and NLP work</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Dev 2</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>Dev 3 — Troy (Data &amp; Infrastructure)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Webhook Integrations: Add Slack and email notification delivery for scan events (WBS 6.3)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Dev 3</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Wire OpenClaw agent to automated data collection pipeline per Gurbachan’s directive</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>OpenShell sandbox — blocked on LXC seccomp fix from Gurbachan</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Implement content freshness automation — scheduled updates with timestamps for AI ranking maintenance</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Ensure all backend infrastructure is demo-ready for Invest Ottawa by third week of May</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Prepare demo of document repository + investor form + DynamoDB migration for Tuesday</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Dev 4 — Tabasum (Integrations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Developer API: Add rate limiting dashboard and usage analytics per API key (WBS 6.2 continued)</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Dev 3</t>
-        </is>
-      </c>
-      <c r="B22" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Add "investor" contact option/link at the bottom of the homepage for potential investors</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Dev 3</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Send final email to Gurbachan (CC Paul) re: OpenClaw/OpenShell Podman UDP socket permission issue</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Dev 3</t>
-        </is>
-      </c>
-      <c r="B24" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>OpenShell sandbox — blocked on LXC seccomp restriction, waiting on Gurbachan</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Dev 3</t>
-        </is>
-      </c>
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Research Amazon H100/H200 accelerator pricing and develop a usage plan for the team’s tiered job system</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Dev 3</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>Dev 4 — Tabasum (Integrations)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Social media API integration: Connect live platform accounts for end-to-end posting (WBS 3.4 continued)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Dev 4</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Monitor website traffic and implement visitor tracking via cookies — report visitor numbers</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Continue creating engaging social media images/videos — use Pexel for images, Synthesia for lip-sync videos</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Approach Algonquin College to explore partnership/advertising collaboration and offer free SEO services</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Create more creative templates with clear text, animated/lady-led content for better engagement</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Prepare social media pipeline and visitor tracking for Invest Ottawa demo by third week of May</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>Dev 5 — Amira (Frontend &amp; UX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Dev 5</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Social media API integration: Connect Buffer/Postiz publishers to live platform accounts and test end-to-end posting (WBS 3.4 — platform adapter)</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Dev 4</t>
-        </is>
-      </c>
-      <c r="B30" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Modify website email capture prompt — emphasize "free analysis" instead of "starter kit", list AEO/GEO before SEO</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Dev 4</t>
-        </is>
-      </c>
-      <c r="B31" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Send Paul email requesting SES SMTP permissions and additional credentials for marketing email</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Dev 4</t>
-        </is>
-      </c>
-      <c r="B32" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Dev 4</t>
-        </is>
-      </c>
-      <c r="B33" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Collaborate with Deepthi, Amira, Samarveer on accelerator usage plan and recommendations for Gurbachan</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Dev 4</t>
-        </is>
-      </c>
-      <c r="B34" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="20" t="inlineStr">
-        <is>
-          <t>Dev 5 — Amira (Frontend &amp; UX)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Multi-Site Dashboard: Begin agency view with bulk operations for multiple sites (WBS 6.1)</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B37" s="21" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Basic Dashboard: Add score trend chart showing historical audit scores over time (WBS 2.3 continued)</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Continue developing main landing page — highly user-friendly, engaging, clear CTAs, email capture</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B38" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Update before/after scan comparison tool — display highest changes at the top per Gurbachan</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="B39" s="31" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Share competitor website example with team for UI/UX inspiration</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B39" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Wire Documents tab to live API endpoints (backend is deployed and matching your schema)</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="B40" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Collaborate with Cairo to optimize main page for user engagement and conversion — debate best email collection approach</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
-        <is>
-          <t>Cleanup</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Wire PDF email gate to POST /api/collect-email endpoint (live on Lambda)</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="B41" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Research and implement daily content creation tools with time-stamped freshness for AI rankings (with Deepthi)</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Dev 5</t>
         </is>
       </c>
-      <c r="B41" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Research Amazon H100/H200 GPU accelerators — evaluate pricing and identify useful tasks from your workload</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Dev 5</t>
-        </is>
-      </c>
-      <c r="B42" s="23" t="inlineStr">
-        <is>
-          <t>Zoom</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Update shared Excel spreadsheet with task status; if blocked, add a note with the reason</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Have front-end prototype application ready for Invest Ottawa demo by third week of May</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>

</xml_diff>